<commit_message>
Vena har fået fjernet igangværende testforløb for RUC10, REF10 og DIS10
</commit_message>
<xml_diff>
--- a/html/Lægesystemer - modtage_excel.XLSX
+++ b/html/Lægesystemer - modtage_excel.XLSX
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC26AFAB-08E9-4A8B-A76D-461D1E34F8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF44D1BE-7652-4DAD-9DC2-3B55E0E680BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Opdateret d. 11-03-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Lægesystemer___modtage">'Opdateret d. 11-03-2026'!$A$1:$K$41</definedName>
+    <definedName name="Lægesystemer___modtage">'Opdateret d. 11-03-2026'!$A$1:$K$40</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="90">
   <si>
     <t>Standard</t>
   </si>
@@ -240,12 +240,6 @@
   </si>
   <si>
     <t>REF06 (H0631R)</t>
-  </si>
-  <si>
-    <t>Psykologhenvisning</t>
-  </si>
-  <si>
-    <t>REF10 (H1031R)</t>
   </si>
   <si>
     <t>Laboratoriesvar</t>
@@ -641,7 +635,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:K40"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -1586,8 +1580,29 @@
       <c r="C32" t="s">
         <v>13</v>
       </c>
+      <c r="D32" t="s">
+        <v>14</v>
+      </c>
+      <c r="E32" t="s">
+        <v>17</v>
+      </c>
+      <c r="F32" t="s">
+        <v>14</v>
+      </c>
+      <c r="G32" t="s">
+        <v>14</v>
+      </c>
+      <c r="H32" t="s">
+        <v>14</v>
+      </c>
       <c r="I32" t="s">
-        <v>20</v>
+        <v>14</v>
+      </c>
+      <c r="J32" t="s">
+        <v>14</v>
+      </c>
+      <c r="K32" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.3">
@@ -1615,9 +1630,6 @@
       <c r="H33" t="s">
         <v>14</v>
       </c>
-      <c r="I33" t="s">
-        <v>14</v>
-      </c>
       <c r="J33" t="s">
         <v>14</v>
       </c>
@@ -1650,6 +1662,9 @@
       <c r="H34" t="s">
         <v>14</v>
       </c>
+      <c r="I34" t="s">
+        <v>14</v>
+      </c>
       <c r="J34" t="s">
         <v>14</v>
       </c>
@@ -1702,28 +1717,7 @@
       <c r="C36" t="s">
         <v>13</v>
       </c>
-      <c r="D36" t="s">
-        <v>14</v>
-      </c>
-      <c r="E36" t="s">
-        <v>17</v>
-      </c>
-      <c r="F36" t="s">
-        <v>14</v>
-      </c>
-      <c r="G36" t="s">
-        <v>14</v>
-      </c>
-      <c r="H36" t="s">
-        <v>14</v>
-      </c>
       <c r="I36" t="s">
-        <v>14</v>
-      </c>
-      <c r="J36" t="s">
-        <v>14</v>
-      </c>
-      <c r="K36" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1737,7 +1731,28 @@
       <c r="C37" t="s">
         <v>13</v>
       </c>
+      <c r="D37" t="s">
+        <v>14</v>
+      </c>
+      <c r="E37" t="s">
+        <v>17</v>
+      </c>
+      <c r="F37" t="s">
+        <v>14</v>
+      </c>
+      <c r="G37" t="s">
+        <v>14</v>
+      </c>
+      <c r="H37" t="s">
+        <v>14</v>
+      </c>
       <c r="I37" t="s">
+        <v>14</v>
+      </c>
+      <c r="J37" t="s">
+        <v>14</v>
+      </c>
+      <c r="K37" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1789,19 +1804,10 @@
       <c r="D39" t="s">
         <v>14</v>
       </c>
-      <c r="E39" t="s">
-        <v>17</v>
-      </c>
       <c r="F39" t="s">
         <v>14</v>
       </c>
-      <c r="G39" t="s">
-        <v>14</v>
-      </c>
       <c r="H39" t="s">
-        <v>14</v>
-      </c>
-      <c r="I39" t="s">
         <v>14</v>
       </c>
       <c r="J39" t="s">
@@ -1824,51 +1830,25 @@
       <c r="D40" t="s">
         <v>14</v>
       </c>
+      <c r="E40" t="s">
+        <v>17</v>
+      </c>
       <c r="F40" t="s">
         <v>14</v>
       </c>
+      <c r="G40" t="s">
+        <v>14</v>
+      </c>
       <c r="H40" t="s">
         <v>14</v>
       </c>
+      <c r="I40" t="s">
+        <v>14</v>
+      </c>
       <c r="J40" t="s">
         <v>14</v>
       </c>
       <c r="K40" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>90</v>
-      </c>
-      <c r="B41" t="s">
-        <v>91</v>
-      </c>
-      <c r="C41" t="s">
-        <v>13</v>
-      </c>
-      <c r="D41" t="s">
-        <v>14</v>
-      </c>
-      <c r="E41" t="s">
-        <v>17</v>
-      </c>
-      <c r="F41" t="s">
-        <v>14</v>
-      </c>
-      <c r="G41" t="s">
-        <v>14</v>
-      </c>
-      <c r="H41" t="s">
-        <v>14</v>
-      </c>
-      <c r="I41" t="s">
-        <v>14</v>
-      </c>
-      <c r="J41" t="s">
-        <v>14</v>
-      </c>
-      <c r="K41" t="s">
         <v>14</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Vena har fået status Tester for afsendelse af DIS13 og afsendelse og modtage for DIS90
</commit_message>
<xml_diff>
--- a/html/Lægesystemer - modtage_excel.XLSX
+++ b/html/Lægesystemer - modtage_excel.XLSX
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DDBB6F6-D1C2-4CEC-AB46-459D319896C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F62A3CD7-1CF0-455A-9872-EEFC4D973C8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="92">
   <si>
     <t>Standard</t>
   </si>
@@ -1317,6 +1317,9 @@
       <c r="H21" t="s">
         <v>15</v>
       </c>
+      <c r="I21" t="s">
+        <v>21</v>
+      </c>
       <c r="J21" t="s">
         <v>15</v>
       </c>

</xml_diff>

<commit_message>
Vena [Psykolog] har fået tilføjet status Tester for REF10, DIS10 og RUC10
</commit_message>
<xml_diff>
--- a/html/Lægesystemer - modtage_excel.XLSX
+++ b/html/Lægesystemer - modtage_excel.XLSX
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Godkendelsesdatabase\GodkendteSystemer\html\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C8A3534-FEC2-4E51-8D7E-773D83128737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4BC32A4-5EA9-468E-A8F8-EF482A9636DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="Opdateret d. 09-09-2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="Lægesystemer___modtage">'Opdateret d. 09-09-2026'!$A$1:$M$50</definedName>
+    <definedName name="Lægesystemer___modtage">'Opdateret d. 09-09-2026'!$A$1:$M$49</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="463" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="459" uniqueCount="108">
   <si>
     <t>Standard</t>
   </si>
@@ -251,12 +251,6 @@
   </si>
   <si>
     <t>REF06 (H0631R)</t>
-  </si>
-  <si>
-    <t>Psykologhenvisning</t>
-  </si>
-  <si>
-    <t>REF10 (H1031R)</t>
   </si>
   <si>
     <t>Laboratoriesvar</t>
@@ -694,7 +688,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
@@ -1761,8 +1755,35 @@
       <c r="C33" t="s">
         <v>15</v>
       </c>
+      <c r="D33" t="s">
+        <v>16</v>
+      </c>
+      <c r="E33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F33" t="s">
+        <v>20</v>
+      </c>
+      <c r="G33" t="s">
+        <v>16</v>
+      </c>
+      <c r="H33" t="s">
+        <v>16</v>
+      </c>
+      <c r="I33" t="s">
+        <v>16</v>
+      </c>
       <c r="J33" t="s">
-        <v>17</v>
+        <v>16</v>
+      </c>
+      <c r="K33" t="s">
+        <v>16</v>
+      </c>
+      <c r="L33" t="s">
+        <v>16</v>
+      </c>
+      <c r="M33" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
@@ -1778,9 +1799,6 @@
       <c r="D34" t="s">
         <v>16</v>
       </c>
-      <c r="E34" t="s">
-        <v>17</v>
-      </c>
       <c r="F34" t="s">
         <v>20</v>
       </c>
@@ -1793,13 +1811,7 @@
       <c r="I34" t="s">
         <v>16</v>
       </c>
-      <c r="J34" t="s">
-        <v>16</v>
-      </c>
       <c r="K34" t="s">
-        <v>16</v>
-      </c>
-      <c r="L34" t="s">
         <v>16</v>
       </c>
       <c r="M34" t="s">
@@ -1819,6 +1831,9 @@
       <c r="D35" t="s">
         <v>16</v>
       </c>
+      <c r="E35" t="s">
+        <v>17</v>
+      </c>
       <c r="F35" t="s">
         <v>20</v>
       </c>
@@ -1831,7 +1846,13 @@
       <c r="I35" t="s">
         <v>16</v>
       </c>
+      <c r="J35" t="s">
+        <v>16</v>
+      </c>
       <c r="K35" t="s">
+        <v>16</v>
+      </c>
+      <c r="L35" t="s">
         <v>16</v>
       </c>
       <c r="M35" t="s">
@@ -1889,54 +1910,27 @@
       <c r="C37" t="s">
         <v>15</v>
       </c>
-      <c r="D37" t="s">
-        <v>16</v>
-      </c>
       <c r="E37" t="s">
         <v>17</v>
-      </c>
-      <c r="F37" t="s">
-        <v>20</v>
-      </c>
-      <c r="G37" t="s">
-        <v>16</v>
-      </c>
-      <c r="H37" t="s">
-        <v>16</v>
-      </c>
-      <c r="I37" t="s">
-        <v>16</v>
-      </c>
-      <c r="J37" t="s">
-        <v>16</v>
-      </c>
-      <c r="K37" t="s">
-        <v>16</v>
-      </c>
-      <c r="L37" t="s">
-        <v>16</v>
-      </c>
-      <c r="M37" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
+        <v>84</v>
+      </c>
+      <c r="B38" t="s">
         <v>86</v>
       </c>
-      <c r="B38" t="s">
-        <v>87</v>
-      </c>
       <c r="C38" t="s">
         <v>15</v>
       </c>
-      <c r="E38" t="s">
-        <v>17</v>
+      <c r="J38" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B39" t="s">
         <v>88</v>
@@ -1944,8 +1938,8 @@
       <c r="C39" t="s">
         <v>15</v>
       </c>
-      <c r="J39" t="s">
-        <v>16</v>
+      <c r="E39" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.3">
@@ -2000,48 +1994,48 @@
       <c r="C43" t="s">
         <v>15</v>
       </c>
-      <c r="E43" t="s">
-        <v>17</v>
+      <c r="D43" t="s">
+        <v>16</v>
+      </c>
+      <c r="F43" t="s">
+        <v>20</v>
+      </c>
+      <c r="G43" t="s">
+        <v>16</v>
+      </c>
+      <c r="H43" t="s">
+        <v>16</v>
+      </c>
+      <c r="I43" t="s">
+        <v>16</v>
+      </c>
+      <c r="J43" t="s">
+        <v>16</v>
+      </c>
+      <c r="K43" t="s">
+        <v>16</v>
+      </c>
+      <c r="M43" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
+        <v>95</v>
+      </c>
+      <c r="B44" t="s">
         <v>97</v>
       </c>
-      <c r="B44" t="s">
-        <v>98</v>
-      </c>
       <c r="C44" t="s">
         <v>15</v>
       </c>
-      <c r="D44" t="s">
-        <v>16</v>
-      </c>
-      <c r="F44" t="s">
-        <v>20</v>
-      </c>
-      <c r="G44" t="s">
-        <v>16</v>
-      </c>
-      <c r="H44" t="s">
-        <v>16</v>
-      </c>
-      <c r="I44" t="s">
-        <v>16</v>
-      </c>
-      <c r="J44" t="s">
-        <v>16</v>
-      </c>
-      <c r="K44" t="s">
-        <v>16</v>
-      </c>
-      <c r="M44" t="s">
-        <v>16</v>
+      <c r="E44" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B45" t="s">
         <v>99</v>
@@ -2049,8 +2043,32 @@
       <c r="C45" t="s">
         <v>15</v>
       </c>
+      <c r="D45" t="s">
+        <v>16</v>
+      </c>
       <c r="E45" t="s">
         <v>17</v>
+      </c>
+      <c r="F45" t="s">
+        <v>20</v>
+      </c>
+      <c r="G45" t="s">
+        <v>16</v>
+      </c>
+      <c r="H45" t="s">
+        <v>16</v>
+      </c>
+      <c r="I45" t="s">
+        <v>16</v>
+      </c>
+      <c r="J45" t="s">
+        <v>16</v>
+      </c>
+      <c r="K45" t="s">
+        <v>16</v>
+      </c>
+      <c r="M45" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.3">
@@ -2066,22 +2084,10 @@
       <c r="D46" t="s">
         <v>16</v>
       </c>
-      <c r="E46" t="s">
-        <v>17</v>
-      </c>
-      <c r="F46" t="s">
-        <v>20</v>
-      </c>
       <c r="G46" t="s">
         <v>16</v>
       </c>
-      <c r="H46" t="s">
-        <v>16</v>
-      </c>
       <c r="I46" t="s">
-        <v>16</v>
-      </c>
-      <c r="J46" t="s">
         <v>16</v>
       </c>
       <c r="K46" t="s">
@@ -2101,19 +2107,7 @@
       <c r="C47" t="s">
         <v>15</v>
       </c>
-      <c r="D47" t="s">
-        <v>16</v>
-      </c>
-      <c r="G47" t="s">
-        <v>16</v>
-      </c>
-      <c r="I47" t="s">
-        <v>16</v>
-      </c>
-      <c r="K47" t="s">
-        <v>16</v>
-      </c>
-      <c r="M47" t="s">
+      <c r="L47" t="s">
         <v>16</v>
       </c>
     </row>
@@ -2141,48 +2135,34 @@
       <c r="C49" t="s">
         <v>15</v>
       </c>
+      <c r="D49" t="s">
+        <v>16</v>
+      </c>
+      <c r="E49" t="s">
+        <v>17</v>
+      </c>
+      <c r="F49" t="s">
+        <v>20</v>
+      </c>
+      <c r="G49" t="s">
+        <v>16</v>
+      </c>
+      <c r="H49" t="s">
+        <v>16</v>
+      </c>
+      <c r="I49" t="s">
+        <v>16</v>
+      </c>
+      <c r="J49" t="s">
+        <v>16</v>
+      </c>
+      <c r="K49" t="s">
+        <v>16</v>
+      </c>
       <c r="L49" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A50" t="s">
-        <v>108</v>
-      </c>
-      <c r="B50" t="s">
-        <v>109</v>
-      </c>
-      <c r="C50" t="s">
-        <v>15</v>
-      </c>
-      <c r="D50" t="s">
-        <v>16</v>
-      </c>
-      <c r="E50" t="s">
-        <v>17</v>
-      </c>
-      <c r="F50" t="s">
-        <v>20</v>
-      </c>
-      <c r="G50" t="s">
-        <v>16</v>
-      </c>
-      <c r="H50" t="s">
-        <v>16</v>
-      </c>
-      <c r="I50" t="s">
-        <v>16</v>
-      </c>
-      <c r="J50" t="s">
-        <v>16</v>
-      </c>
-      <c r="K50" t="s">
-        <v>16</v>
-      </c>
-      <c r="L50" t="s">
-        <v>16</v>
-      </c>
-      <c r="M50" t="s">
+      <c r="M49" t="s">
         <v>16</v>
       </c>
     </row>

</xml_diff>